<commit_message>
Fixed labels in week 9 slides
</commit_message>
<xml_diff>
--- a/Homework 3/Homework 3 data.xlsx
+++ b/Homework 3/Homework 3 data.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -55,7 +55,7 @@
   <fonts count="5">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -78,7 +78,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -166,23 +166,198 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1f497d"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="eeece1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4f81bd"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="c0504d"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9bbb59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064a2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4bacc6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="f79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ff"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G181"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.7" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.95"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -205,7 +380,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
         <v>39814</v>
       </c>
@@ -228,7 +403,7 @@
         <v>-0.0127620783956245</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>39845</v>
       </c>
@@ -251,7 +426,7 @@
         <v>-0.0240073868882733</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>39873</v>
       </c>
@@ -274,7 +449,7 @@
         <v>-0.0300806945294674</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>39904</v>
       </c>
@@ -297,7 +472,7 @@
         <v>-0.0292968750000001</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>39934</v>
       </c>
@@ -305,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0.056176982351479</v>
+        <v>0.0561769823514791</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0.0291574502312488</v>
@@ -320,7 +495,7 @@
         <v>-0.0150905432595574</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>39965</v>
       </c>
@@ -328,7 +503,7 @@
         <v>0.0001</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>0.00219960160119847</v>
+        <v>0.00219960160119848</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>0.0504103165298944</v>
@@ -343,7 +518,7 @@
         <v>0.0143003064351379</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>39995</v>
       </c>
@@ -366,7 +541,7 @@
         <v>-0.013091641490433</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>40026</v>
       </c>
@@ -389,7 +564,7 @@
         <v>-0.00102040816326543</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>40057</v>
       </c>
@@ -400,7 +575,7 @@
         <v>0.0371678959247073</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>0.0305449496702534</v>
+        <v>0.0305449496702535</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0.00806596400811088</v>
@@ -412,7 +587,7 @@
         <v>-0.00817160367722147</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>40087</v>
       </c>
@@ -435,7 +610,7 @@
         <v>-0.00102986611740485</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>40118</v>
       </c>
@@ -455,10 +630,10 @@
         <v>0.00659646887159537</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>-0.00206185567010308</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>-0.00206185567010309</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>40148</v>
       </c>
@@ -481,7 +656,7 @@
         <v>0.00309917355371914</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>40179</v>
       </c>
@@ -504,7 +679,7 @@
         <v>0.00102986611740463</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>40210</v>
       </c>
@@ -527,7 +702,7 @@
         <v>0.0133744855967077</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
         <v>40238</v>
       </c>
@@ -550,7 +725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
         <v>40269</v>
       </c>
@@ -573,7 +748,7 @@
         <v>-0.00710659898477162</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
         <v>40299</v>
       </c>
@@ -596,7 +771,7 @@
         <v>0.00817995910020453</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>40330</v>
       </c>
@@ -619,7 +794,7 @@
         <v>-0.00811359026369174</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <v>40360</v>
       </c>
@@ -642,7 +817,7 @@
         <v>0.00306748466257689</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>40391</v>
       </c>
@@ -665,7 +840,7 @@
         <v>-0.0122324159021408</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
         <v>40422</v>
       </c>
@@ -673,7 +848,7 @@
         <v>0.0001</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>0.0891889591585075</v>
+        <v>0.0891889591585076</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>0.0954861111111112</v>
@@ -688,7 +863,7 @@
         <v>0.00928792569659431</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
         <v>40452</v>
       </c>
@@ -711,7 +886,7 @@
         <v>0.00204498977505119</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
         <v>40483</v>
       </c>
@@ -734,7 +909,7 @@
         <v>0.00612244897959169</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
         <v>40513</v>
       </c>
@@ -757,7 +932,7 @@
         <v>-0.0253549695740365</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
         <v>40544</v>
       </c>
@@ -765,7 +940,7 @@
         <v>0.0001</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>0.0235710585391124</v>
+        <v>0.0235710585391125</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>-0.00495554583879909</v>
@@ -777,10 +952,10 @@
         <v>0.00388346487006741</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>0.00312174817898025</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.00312174817898026</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>40575</v>
       </c>
@@ -803,7 +978,7 @@
         <v>0.0134854771784232</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
         <v>40603</v>
       </c>
@@ -826,7 +1001,7 @@
         <v>0.0245649948822928</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
         <v>40634</v>
       </c>
@@ -849,7 +1024,7 @@
         <v>0.00599400599400601</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>40664</v>
       </c>
@@ -872,7 +1047,7 @@
         <v>0.000993048659384321</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
         <v>40695</v>
       </c>
@@ -895,7 +1070,7 @@
         <v>0.0238095238095237</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <v>40725</v>
       </c>
@@ -912,13 +1087,13 @@
         <v>-0.0144230769230769</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>0.00320918095238087</v>
+        <v>0.00320918095238088</v>
       </c>
       <c r="G32" s="1" t="n">
         <v>-0.00290697674418616</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
         <v>40756</v>
       </c>
@@ -941,7 +1116,7 @@
         <v>0.0155490767735667</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <v>40787</v>
       </c>
@@ -961,10 +1136,10 @@
         <v>-0.0150406985645933</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>-0.0114832535885166</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>-0.0114832535885167</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
         <v>40817</v>
       </c>
@@ -987,7 +1162,7 @@
         <v>0.00871248789932233</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
         <v>40848</v>
       </c>
@@ -1010,7 +1185,7 @@
         <v>0.000959692898272468</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
         <v>40878</v>
       </c>
@@ -1033,7 +1208,7 @@
         <v>-0.00671140939597315</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
         <v>40909</v>
       </c>
@@ -1056,7 +1231,7 @@
         <v>0.00193050193050204</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
         <v>40940</v>
       </c>
@@ -1079,7 +1254,7 @@
         <v>0.00674373795761074</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
         <v>40969</v>
       </c>
@@ -1099,10 +1274,10 @@
         <v>0.000216554702495264</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>-0.00287081339712913</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>-0.00287081339712914</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="n">
         <v>41000</v>
       </c>
@@ -1125,7 +1300,7 @@
         <v>-0.010556621880998</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="n">
         <v>41030</v>
       </c>
@@ -1148,7 +1323,7 @@
         <v>-0.0116391852570321</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="n">
         <v>41061</v>
       </c>
@@ -1171,7 +1346,7 @@
         <v>0.00588812561334651</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="n">
         <v>41091</v>
       </c>
@@ -1191,10 +1366,10 @@
         <v>0.0110983015267174</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>0.024390243902439</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.0243902439024391</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="n">
         <v>41122</v>
       </c>
@@ -1217,7 +1392,7 @@
         <v>-0.0114285714285713</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="n">
         <v>41153</v>
       </c>
@@ -1240,7 +1415,7 @@
         <v>-0.0134874759152216</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="n">
         <v>41183</v>
       </c>
@@ -1263,7 +1438,7 @@
         <v>-0.00390625000000011</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="n">
         <v>41214</v>
       </c>
@@ -1286,7 +1461,7 @@
         <v>0.00588235294117645</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="n">
         <v>41244</v>
       </c>
@@ -1309,7 +1484,7 @@
         <v>-0.00535197296330903</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="n">
         <v>41275</v>
       </c>
@@ -1332,7 +1507,7 @@
         <v>0.0137795275590551</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="n">
         <v>41306</v>
       </c>
@@ -1355,7 +1530,7 @@
         <v>0.00582524271844642</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
         <v>41334</v>
       </c>
@@ -1378,7 +1553,7 @@
         <v>0.00994153231748673</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
         <v>41365</v>
       </c>
@@ -1401,7 +1576,7 @@
         <v>0.00382409177820264</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
         <v>41395</v>
       </c>
@@ -1424,7 +1599,7 @@
         <v>0.00952380952380949</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="n">
         <v>41426</v>
       </c>
@@ -1447,7 +1622,7 @@
         <v>0.00283018867924545</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="n">
         <v>41456</v>
       </c>
@@ -1461,7 +1636,7 @@
         <v>0.15810386250231</v>
       </c>
       <c r="E56" s="1" t="n">
-        <v>0.0392687880839539</v>
+        <v>0.039268788083954</v>
       </c>
       <c r="F56" s="1" t="n">
         <v>0.00418866341463398</v>
@@ -1470,7 +1645,7 @@
         <v>0.000940733772342384</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="n">
         <v>41487</v>
       </c>
@@ -1490,10 +1665,10 @@
         <v>-0.00482097276264581</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>-0.0131578947368421</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>-0.0131578947368422</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="n">
         <v>41518</v>
       </c>
@@ -1516,7 +1691,7 @@
         <v>0.00857142857142845</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="n">
         <v>41548</v>
       </c>
@@ -1539,7 +1714,7 @@
         <v>0.0292728989612843</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="n">
         <v>41579</v>
       </c>
@@ -1562,7 +1737,7 @@
         <v>0.0110091743119265</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="n">
         <v>41609</v>
       </c>
@@ -1585,7 +1760,7 @@
         <v>0.000907441016333888</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="n">
         <v>41640</v>
       </c>
@@ -1602,13 +1777,13 @@
         <v>0.0220883534136547</v>
       </c>
       <c r="F62" s="1" t="n">
-        <v>0.00229963213939976</v>
+        <v>0.00229963213939977</v>
       </c>
       <c r="G62" s="1" t="n">
         <v>-0.00181323662737987</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="n">
         <v>41671</v>
       </c>
@@ -1631,7 +1806,7 @@
         <v>0.0108991825613081</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="n">
         <v>41699</v>
       </c>
@@ -1645,7 +1820,7 @@
         <v>-0.106053825992457</v>
       </c>
       <c r="E64" s="1" t="n">
-        <v>0.0258574532253923</v>
+        <v>0.0258574532253924</v>
       </c>
       <c r="F64" s="1" t="n">
         <v>-0.00458665384615387</v>
@@ -1654,7 +1829,7 @@
         <v>0.0188679245283019</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="n">
         <v>41730</v>
       </c>
@@ -1665,7 +1840,7 @@
         <v>0.00724091988646247</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>-0.0756578947368421</v>
+        <v>-0.0756578947368422</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>0.0360024829298573</v>
@@ -1677,7 +1852,7 @@
         <v>0.00617283950617287</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="n">
         <v>41760</v>
       </c>
@@ -1688,7 +1863,7 @@
         <v>0.0233494363929148</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>0.0285471143431843</v>
+        <v>0.0285471143431844</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0.000599161174355878</v>
@@ -1700,7 +1875,7 @@
         <v>0.00964066608238379</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="n">
         <v>41791</v>
       </c>
@@ -1723,7 +1898,7 @@
         <v>-0.015625</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="n">
         <v>41821</v>
       </c>
@@ -1731,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>-0.013880440192446</v>
+        <v>-0.0138804401924461</v>
       </c>
       <c r="D68" s="1" t="n">
         <v>-0.00972559916637705</v>
@@ -1746,7 +1921,7 @@
         <v>0.00881834215167543</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="n">
         <v>41852</v>
       </c>
@@ -1769,7 +1944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="n">
         <v>41883</v>
       </c>
@@ -1783,7 +1958,7 @@
         <v>-0.0194821361882236</v>
       </c>
       <c r="E70" s="1" t="n">
-        <v>-0.030078030170479</v>
+        <v>-0.0300780301704791</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>-0.00397203864734275</v>
@@ -1792,7 +1967,7 @@
         <v>0.000874125874125831</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="n">
         <v>41913</v>
       </c>
@@ -1815,7 +1990,7 @@
         <v>-0.00174672489082961</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="n">
         <v>41944</v>
       </c>
@@ -1838,7 +2013,7 @@
         <v>0.00874890638670167</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="n">
         <v>41974</v>
       </c>
@@ -1861,7 +2036,7 @@
         <v>-0.00260190806591498</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="n">
         <v>42005</v>
       </c>
@@ -1875,7 +2050,7 @@
         <v>0.0550513139941864</v>
       </c>
       <c r="E74" s="1" t="n">
-        <v>0.0185915492957744</v>
+        <v>0.0185915492957745</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>0.00285390438247024</v>
@@ -1884,7 +2059,7 @@
         <v>0.011304347826087</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="n">
         <v>42036</v>
       </c>
@@ -1907,7 +2082,7 @@
         <v>-0.0206362854686156</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="n">
         <v>42064</v>
       </c>
@@ -1924,13 +2099,13 @@
         <v>-0.0101112243282133</v>
       </c>
       <c r="F76" s="1" t="n">
-        <v>-7.7049504950577E-005</v>
+        <v>-7.70495049505771E-005</v>
       </c>
       <c r="G76" s="1" t="n">
         <v>0.0114135206321333</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="n">
         <v>42095</v>
       </c>
@@ -1953,7 +2128,7 @@
         <v>-0.0121527777777777</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="n">
         <v>42125</v>
       </c>
@@ -1976,7 +2151,7 @@
         <v>0.00790861159929701</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="n">
         <v>42156</v>
       </c>
@@ -1999,7 +2174,7 @@
         <v>-0.00871839581517009</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="n">
         <v>42186</v>
       </c>
@@ -2022,7 +2197,7 @@
         <v>0.0255057167985928</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="n">
         <v>42217</v>
       </c>
@@ -2045,7 +2220,7 @@
         <v>-0.00600343053173247</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="n">
         <v>42248</v>
       </c>
@@ -2068,7 +2243,7 @@
         <v>0.0500431406384814</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="n">
         <v>42278</v>
       </c>
@@ -2091,7 +2266,7 @@
         <v>-0.00493015612161052</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="n">
         <v>42309</v>
       </c>
@@ -2114,7 +2289,7 @@
         <v>-0.00660611065235339</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="n">
         <v>42339</v>
       </c>
@@ -2137,7 +2312,7 @@
         <v>0.00847921518517758</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="n">
         <v>42370</v>
       </c>
@@ -2160,7 +2335,7 @@
         <v>0.0123660346248968</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="n">
         <v>42401</v>
       </c>
@@ -2171,7 +2346,7 @@
         <v>-0.00145170295924058</v>
       </c>
       <c r="D87" s="1" t="n">
-        <v>-0.0636998254799302</v>
+        <v>-0.0636998254799303</v>
       </c>
       <c r="E87" s="1" t="n">
         <v>0.0218204488778055</v>
@@ -2183,7 +2358,7 @@
         <v>0.0154723127035832</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="n">
         <v>42430</v>
       </c>
@@ -2206,7 +2381,7 @@
         <v>-0.00481154771451486</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="n">
         <v>42461</v>
       </c>
@@ -2229,7 +2404,7 @@
         <v>-0.0177276390008059</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="n">
         <v>42491</v>
       </c>
@@ -2237,7 +2412,7 @@
         <v>0.0001</v>
       </c>
       <c r="C90" s="1" t="n">
-        <v>0.0178290508652334</v>
+        <v>0.0178290508652335</v>
       </c>
       <c r="D90" s="1" t="n">
         <v>0.0598423968167279</v>
@@ -2252,7 +2427,7 @@
         <v>-0.018047579983593</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="n">
         <v>42522</v>
       </c>
@@ -2269,13 +2444,13 @@
         <v>0.0727728418632414</v>
       </c>
       <c r="F91" s="1" t="n">
-        <v>0.0019810931174089</v>
+        <v>0.00198109311740891</v>
       </c>
       <c r="G91" s="1" t="n">
         <v>-0.0125313283208021</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="n">
         <v>42552</v>
       </c>
@@ -2298,7 +2473,7 @@
         <v>0.00676818950930636</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="n">
         <v>42583</v>
       </c>
@@ -2321,7 +2496,7 @@
         <v>-0.0201680672268908</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="n">
         <v>42614</v>
       </c>
@@ -2344,7 +2519,7 @@
         <v>0.00514579759862777</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="n">
         <v>42644</v>
       </c>
@@ -2367,7 +2542,7 @@
         <v>0.006825938566553</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="n">
         <v>42675</v>
       </c>
@@ -2390,7 +2565,7 @@
         <v>0.0406779661016947</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="n">
         <v>42705</v>
       </c>
@@ -2413,7 +2588,7 @@
         <v>0.0127819297047391</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="n">
         <v>42736</v>
       </c>
@@ -2436,7 +2611,7 @@
         <v>-0.0177562550443907</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="n">
         <v>42767</v>
       </c>
@@ -2459,7 +2634,7 @@
         <v>-0.0024650780608052</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="n">
         <v>42795</v>
       </c>
@@ -2482,7 +2657,7 @@
         <v>-0.00408553038471426</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="n">
         <v>42826</v>
       </c>
@@ -2505,7 +2680,7 @@
         <v>-0.000827129859387932</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="n">
         <v>42856</v>
       </c>
@@ -2528,7 +2703,7 @@
         <v>-0.021523178807947</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="n">
         <v>42887</v>
       </c>
@@ -2551,7 +2726,7 @@
         <v>0.00169204737732653</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="n">
         <v>42917</v>
       </c>
@@ -2574,7 +2749,7 @@
         <v>0.00929054054054057</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="n">
         <v>42948</v>
       </c>
@@ -2597,7 +2772,7 @@
         <v>-0.0133891213389121</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="n">
         <v>42979</v>
       </c>
@@ -2620,7 +2795,7 @@
         <v>0.000848176420695568</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="n">
         <v>43009</v>
       </c>
@@ -2643,7 +2818,7 @@
         <v>0.00677966101694927</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="n">
         <v>43040</v>
       </c>
@@ -2666,7 +2841,7 @@
         <v>-0.0101010101010102</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="n">
         <v>43070</v>
       </c>
@@ -2689,7 +2864,7 @@
         <v>0.00200578347777469</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="n">
         <v>43101</v>
       </c>
@@ -2712,7 +2887,7 @@
         <v>0.0154373927958833</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="n">
         <v>43132</v>
       </c>
@@ -2735,7 +2910,7 @@
         <v>0.00253378378378377</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="n">
         <v>43160</v>
       </c>
@@ -2743,7 +2918,7 @@
         <v>0.0011</v>
       </c>
       <c r="C112" s="1" t="n">
-        <v>-0.0255152706757727</v>
+        <v>-0.0255152706757728</v>
       </c>
       <c r="D112" s="1" t="n">
         <v>-0.025325474447827</v>
@@ -2758,7 +2933,7 @@
         <v>-0.00274641954507149</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="n">
         <v>43191</v>
       </c>
@@ -2781,7 +2956,7 @@
         <v>-0.0118343195266273</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="n">
         <v>43221</v>
       </c>
@@ -2804,7 +2979,7 @@
         <v>0.0205303678357571</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="n">
         <v>43252</v>
       </c>
@@ -2827,7 +3002,7 @@
         <v>-0.0176026823134953</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="n">
         <v>43282</v>
       </c>
@@ -2844,13 +3019,13 @@
         <v>0.0156756756756757</v>
       </c>
       <c r="F116" s="1" t="n">
-        <v>0.00365602261048314</v>
+        <v>0.00365602261048315</v>
       </c>
       <c r="G116" s="1" t="n">
         <v>0.0102389078498293</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="n">
         <v>43313</v>
       </c>
@@ -2858,7 +3033,7 @@
         <v>0.0016</v>
       </c>
       <c r="C117" s="1" t="n">
-        <v>0.0324625432193621</v>
+        <v>0.0324625432193622</v>
       </c>
       <c r="D117" s="1" t="n">
         <v>0.0429721907638103</v>
@@ -2873,7 +3048,7 @@
         <v>0.0185810810810811</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="n">
         <v>43344</v>
       </c>
@@ -2896,7 +3071,7 @@
         <v>-0.0033167495854064</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="n">
         <v>43374</v>
       </c>
@@ -2919,7 +3094,7 @@
         <v>0.00748752079866888</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="n">
         <v>43405</v>
       </c>
@@ -2942,7 +3117,7 @@
         <v>-0.0363336085879438</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="n">
         <v>43435</v>
       </c>
@@ -2950,10 +3125,10 @@
         <v>0.002</v>
       </c>
       <c r="C121" s="1" t="n">
-        <v>-0.0904014174392534</v>
+        <v>-0.0904014174392535</v>
       </c>
       <c r="D121" s="1" t="n">
-        <v>-0.120915070257018</v>
+        <v>-0.120915070257019</v>
       </c>
       <c r="E121" s="1" t="n">
         <v>-0.0707818688763811</v>
@@ -2965,7 +3140,7 @@
         <v>0.00445691600704667</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="n">
         <v>43466</v>
       </c>
@@ -2988,7 +3163,7 @@
         <v>-0.023235800344234</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="n">
         <v>43497</v>
       </c>
@@ -2996,7 +3171,7 @@
         <v>0.0018</v>
       </c>
       <c r="C123" s="1" t="n">
-        <v>0.032005120819331</v>
+        <v>0.0320051208193311</v>
       </c>
       <c r="D123" s="1" t="n">
         <v>0.0494092373791621</v>
@@ -3011,7 +3186,7 @@
         <v>-0.00881057268722463</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="n">
         <v>43525</v>
       </c>
@@ -3034,7 +3209,7 @@
         <v>-0.0213066666666667</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="n">
         <v>43556</v>
       </c>
@@ -3057,7 +3232,7 @@
         <v>-0.0218181818181819</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="n">
         <v>43586</v>
       </c>
@@ -3080,7 +3255,7 @@
         <v>-0.0195167286245352</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="n">
         <v>43617</v>
       </c>
@@ -3103,7 +3278,7 @@
         <v>-0.0161137440758293</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="n">
         <v>43647</v>
       </c>
@@ -3126,7 +3301,7 @@
         <v>0.0154142581888246</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="n">
         <v>43678</v>
       </c>
@@ -3149,7 +3324,7 @@
         <v>0.0113851992409868</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="n">
         <v>43709</v>
       </c>
@@ -3163,7 +3338,7 @@
         <v>-0.0566119901291915</v>
       </c>
       <c r="E130" s="1" t="n">
-        <v>0.0362317851061495</v>
+        <v>0.0362317851061496</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0.00125931979695437</v>
@@ -3172,7 +3347,7 @@
         <v>0.00187617260787998</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="n">
         <v>43739</v>
       </c>
@@ -3195,7 +3370,7 @@
         <v>-0.0102996254681648</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="n">
         <v>43770</v>
       </c>
@@ -3218,7 +3393,7 @@
         <v>-0.00283822138126788</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="n">
         <v>43800</v>
       </c>
@@ -3241,7 +3416,7 @@
         <v>-0.00394960483410389</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="n">
         <v>43831</v>
       </c>
@@ -3264,7 +3439,7 @@
         <v>0.0049067713444555</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="n">
         <v>43862</v>
       </c>
@@ -3287,7 +3462,7 @@
         <v>-0.0341796875</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="n">
         <v>43891</v>
       </c>
@@ -3310,7 +3485,7 @@
         <v>-0.0202912053290126</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="n">
         <v>43922</v>
       </c>
@@ -3324,7 +3499,7 @@
         <v>0.138878377355635</v>
       </c>
       <c r="E137" s="1" t="n">
-        <v>0.0358288770053476</v>
+        <v>0.0358288770053477</v>
       </c>
       <c r="F137" s="1" t="n">
         <v>0.0120024254881808</v>
@@ -3333,7 +3508,7 @@
         <v>0.00206825232678387</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="n">
         <v>43952</v>
       </c>
@@ -3356,7 +3531,7 @@
         <v>-0.0206398348813209</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="n">
         <v>43983</v>
       </c>
@@ -3379,7 +3554,7 @@
         <v>0.017913593256059</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="n">
         <v>44013</v>
       </c>
@@ -3402,7 +3577,7 @@
         <v>0.00931677018633548</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="n">
         <v>44044</v>
       </c>
@@ -3425,7 +3600,7 @@
         <v>-0.0225641025641027</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="n">
         <v>44075</v>
       </c>
@@ -3439,7 +3614,7 @@
         <v>0.0310149828018422</v>
       </c>
       <c r="E142" s="1" t="n">
-        <v>-0.00396623448410915</v>
+        <v>-0.00396623448410916</v>
       </c>
       <c r="F142" s="1" t="n">
         <v>-3.07645875251561E-005</v>
@@ -3448,7 +3623,7 @@
         <v>-0.00944386149003151</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="n">
         <v>44105</v>
       </c>
@@ -3471,7 +3646,7 @@
         <v>-0.0307203389830507</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="n">
         <v>44136</v>
       </c>
@@ -3494,7 +3669,7 @@
         <v>-0.0120218579234974</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="n">
         <v>44166</v>
       </c>
@@ -3508,7 +3683,7 @@
         <v>0.0357007560431712</v>
       </c>
       <c r="E145" s="1" t="n">
-        <v>0.00220129795333745</v>
+        <v>0.00220129795333746</v>
       </c>
       <c r="F145" s="1" t="n">
         <v>0.00169897384305817</v>
@@ -3517,7 +3692,7 @@
         <v>-0.00524466423737646</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="n">
         <v>44197</v>
       </c>
@@ -3540,7 +3715,7 @@
         <v>0.0313199105145414</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="n">
         <v>44228</v>
       </c>
@@ -3563,7 +3738,7 @@
         <v>-0.00759219088937091</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="n">
         <v>44256</v>
       </c>
@@ -3586,7 +3761,7 @@
         <v>0.0459016393442624</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="n">
         <v>44287</v>
       </c>
@@ -3609,7 +3784,7 @@
         <v>-0.00208986415882961</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="n">
         <v>44317</v>
       </c>
@@ -3632,7 +3807,7 @@
         <v>0.032460732984293</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="n">
         <v>44348</v>
       </c>
@@ -3649,13 +3824,13 @@
         <v>-0.0223405256569296</v>
       </c>
       <c r="F151" s="1" t="n">
-        <v>-0.00263065392354111</v>
+        <v>-0.00263065392354112</v>
       </c>
       <c r="G151" s="1" t="n">
         <v>-0.00912778904665312</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="n">
         <v>44378</v>
       </c>
@@ -3678,7 +3853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="n">
         <v>44409</v>
       </c>
@@ -3701,7 +3876,7 @@
         <v>0.0235414534288638</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="n">
         <v>44440</v>
       </c>
@@ -3724,7 +3899,7 @@
         <v>0.0089999999999999</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="n">
         <v>44470</v>
       </c>
@@ -3747,7 +3922,7 @@
         <v>-0.00297324083250738</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="n">
         <v>44501</v>
       </c>
@@ -3770,7 +3945,7 @@
         <v>0.0467196819085487</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="n">
         <v>44531</v>
       </c>
@@ -3793,7 +3968,7 @@
         <v>0.0462949797515417</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="n">
         <v>44562</v>
       </c>
@@ -3816,7 +3991,7 @@
         <v>0.0536363636363637</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="n">
         <v>44593</v>
       </c>
@@ -3839,7 +4014,7 @@
         <v>-0.00949094046591881</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="n">
         <v>44621</v>
       </c>
@@ -3862,7 +4037,7 @@
         <v>0.00087108013937276</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="n">
         <v>44652</v>
       </c>
@@ -3885,7 +4060,7 @@
         <v>0.0426457789382071</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="n">
         <v>44682</v>
       </c>
@@ -3908,7 +4083,7 @@
         <v>0.00751252086811349</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="n">
         <v>44713</v>
       </c>
@@ -3931,7 +4106,7 @@
         <v>-0.0215410107705054</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="n">
         <v>44743</v>
       </c>
@@ -3954,7 +4129,7 @@
         <v>0.00338696020321749</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="n">
         <v>44774</v>
       </c>
@@ -3977,7 +4152,7 @@
         <v>-0.00843881856540085</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="n">
         <v>44805</v>
       </c>
@@ -4000,7 +4175,7 @@
         <v>0.0221276595744682</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="n">
         <v>44835</v>
       </c>
@@ -4023,7 +4198,7 @@
         <v>0.0224812656119899</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="n">
         <v>44866</v>
       </c>
@@ -4046,7 +4221,7 @@
         <v>-0.0130293159609121</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="n">
         <v>44896</v>
       </c>
@@ -4069,7 +4244,7 @@
         <v>0.0299154057166622</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="n">
         <v>44927</v>
       </c>
@@ -4092,7 +4267,7 @@
         <v>-0.0112994350282486</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="n">
         <v>44958</v>
       </c>
@@ -4115,7 +4290,7 @@
         <v>0.0195918367346939</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="n">
         <v>44986</v>
       </c>
@@ -4138,7 +4313,7 @@
         <v>-0.020744536709564</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="n">
         <v>45017</v>
       </c>
@@ -4161,7 +4336,7 @@
         <v>-0.0114472608340148</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="n">
         <v>45047</v>
       </c>
@@ -4184,7 +4359,7 @@
         <v>0.00909842845326714</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="n">
         <v>45078</v>
       </c>
@@ -4207,7 +4382,7 @@
         <v>0.0245901639344264</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="n">
         <v>45108</v>
       </c>
@@ -4230,7 +4405,7 @@
         <v>0.00239999999999996</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="n">
         <v>45139</v>
       </c>
@@ -4253,7 +4428,7 @@
         <v>0.0311252992817239</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="n">
         <v>45170</v>
       </c>
@@ -4276,7 +4451,7 @@
         <v>0.0448916408668731</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="n">
         <v>45200</v>
       </c>
@@ -4299,7 +4474,7 @@
         <v>0.00740740740740731</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="n">
         <v>45231</v>
       </c>
@@ -4313,7 +4488,7 @@
         <v>0.0418176476349035</v>
       </c>
       <c r="E180" s="1" t="n">
-        <v>0.051009564293305</v>
+        <v>0.0510095642933051</v>
       </c>
       <c r="F180" s="1" t="n">
         <v>0.013259557032115</v>
@@ -4322,7 +4497,7 @@
         <v>0.00808823529411784</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="13.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="n">
         <v>45261</v>
       </c>

</xml_diff>